<commit_message>
Slight tweaks to the active attack result XLSX file
</commit_message>
<xml_diff>
--- a/results/0_excel_files/active_attack_results.xlsx
+++ b/results/0_excel_files/active_attack_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Bakalaura Darbs\!Code\Bakalaura_darbs\results\0_excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365F5F48-5AD1-4033-9293-0511485A3C93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB6944-A66A-4166-A5AF-22F5098A6419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1CF9389B-EC12-4777-A84E-B567E82B38F5}"/>
   </bookViews>
@@ -76,10 +76,10 @@
     <t>10_document_inspector_attack</t>
   </si>
   <si>
-    <t>Total attack time lapse (min, sec)</t>
+    <t>Attack time for each stego-file data set (min.sec)</t>
   </si>
   <si>
-    <t>Attack time for each stego-file data set (min, sec)</t>
+    <t>Total attack time lapse (min.sec)</t>
   </si>
 </sst>
 </file>
@@ -814,31 +814,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
@@ -854,6 +836,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1241,656 +1241,656 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15" t="s">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>19</v>
-      </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="11">
         <v>1.05</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="4">
         <v>0.19</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="15"/>
+      <c r="B3" s="12"/>
       <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="15"/>
+      <c r="B4" s="12"/>
       <c r="C4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="12"/>
       <c r="C5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="9">
+      <c r="D5" s="5">
         <v>0.17</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="8"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="12"/>
       <c r="C6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="9">
+      <c r="D6" s="5">
         <v>0.11</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="12" t="s">
+      <c r="A7" s="16"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="7">
         <v>0.16</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="11">
         <v>1.04</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="4">
         <v>0.18</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="3"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="12"/>
       <c r="C9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="9">
+      <c r="D9" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="3"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="12"/>
       <c r="C10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D10" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="8"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="12"/>
       <c r="C11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="5">
         <v>0.16</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="12"/>
       <c r="C12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="5">
         <v>0.11</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="12" t="s">
+      <c r="A13" s="16"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="7">
         <v>0.16</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="11">
         <v>1.05</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="4">
         <v>0.19</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="3"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="12"/>
       <c r="C15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="8"/>
-      <c r="B16" s="3"/>
+      <c r="A16" s="15"/>
+      <c r="B16" s="12"/>
       <c r="C16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="9">
+      <c r="D16" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="8"/>
-      <c r="B17" s="3"/>
+      <c r="A17" s="15"/>
+      <c r="B17" s="12"/>
       <c r="C17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="9">
+      <c r="D17" s="5">
         <v>0.17</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="3"/>
+      <c r="A18" s="15"/>
+      <c r="B18" s="12"/>
       <c r="C18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D18" s="9">
+      <c r="D18" s="5">
         <v>0.11</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12" t="s">
+      <c r="A19" s="16"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D19" s="13">
+      <c r="D19" s="7">
         <v>0.16</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="11">
         <v>5.29</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="4">
         <v>1.34</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="8"/>
-      <c r="B21" s="3"/>
+      <c r="A21" s="15"/>
+      <c r="B21" s="12"/>
       <c r="C21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="8"/>
-      <c r="B22" s="3"/>
+      <c r="A22" s="15"/>
+      <c r="B22" s="12"/>
       <c r="C22" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D22" s="9">
+      <c r="D22" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="8"/>
-      <c r="B23" s="3"/>
+      <c r="A23" s="15"/>
+      <c r="B23" s="12"/>
       <c r="C23" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="5">
         <v>1.31</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="8"/>
-      <c r="B24" s="3"/>
+      <c r="A24" s="15"/>
+      <c r="B24" s="12"/>
       <c r="C24" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D24" s="9">
+      <c r="D24" s="5">
         <v>0.59</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="10"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="12" t="s">
+      <c r="A25" s="16"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D25" s="13">
+      <c r="D25" s="7">
         <v>1.24</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26" s="11">
         <v>15.4</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="4">
         <v>4.2</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-      <c r="B27" s="3"/>
+      <c r="A27" s="15"/>
+      <c r="B27" s="12"/>
       <c r="C27" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D27" s="9">
+      <c r="D27" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="3"/>
+      <c r="A28" s="15"/>
+      <c r="B28" s="12"/>
       <c r="C28" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="8"/>
-      <c r="B29" s="3"/>
+      <c r="A29" s="15"/>
+      <c r="B29" s="12"/>
       <c r="C29" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D29" s="9">
+      <c r="D29" s="5">
         <v>4.18</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="8"/>
-      <c r="B30" s="3"/>
+      <c r="A30" s="15"/>
+      <c r="B30" s="12"/>
       <c r="C30" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D30" s="9">
+      <c r="D30" s="5">
         <v>2.34</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="10"/>
-      <c r="B31" s="11"/>
-      <c r="C31" s="12" t="s">
+      <c r="A31" s="16"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D31" s="13">
+      <c r="D31" s="7">
         <v>4.26</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32" s="11">
         <v>1.1499999999999999</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="4">
         <v>0.23</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="8"/>
-      <c r="B33" s="3"/>
+      <c r="A33" s="15"/>
+      <c r="B33" s="12"/>
       <c r="C33" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D33" s="9">
+      <c r="D33" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="8"/>
-      <c r="B34" s="3"/>
+      <c r="A34" s="15"/>
+      <c r="B34" s="12"/>
       <c r="C34" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D34" s="9">
+      <c r="D34" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="8"/>
-      <c r="B35" s="3"/>
+      <c r="A35" s="15"/>
+      <c r="B35" s="12"/>
       <c r="C35" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D35" s="9">
+      <c r="D35" s="5">
         <v>0.19</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="8"/>
-      <c r="B36" s="3"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="12"/>
       <c r="C36" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D36" s="9">
+      <c r="D36" s="5">
         <v>0.15</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="12" t="s">
+      <c r="A37" s="16"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="13">
+      <c r="D37" s="7">
         <v>0.17</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B38" s="5">
-        <v>0</v>
-      </c>
-      <c r="C38" s="6" t="s">
+      <c r="B38" s="11">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D38" s="7">
+      <c r="D38" s="4">
         <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="8"/>
-      <c r="B39" s="3"/>
+      <c r="A39" s="15"/>
+      <c r="B39" s="12"/>
       <c r="C39" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D39" s="9">
+      <c r="D39" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="8"/>
-      <c r="B40" s="3"/>
+      <c r="A40" s="15"/>
+      <c r="B40" s="12"/>
       <c r="C40" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="8"/>
-      <c r="B41" s="3"/>
+      <c r="A41" s="15"/>
+      <c r="B41" s="12"/>
       <c r="C41" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D41" s="9">
+      <c r="D41" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="8"/>
-      <c r="B42" s="3"/>
+      <c r="A42" s="15"/>
+      <c r="B42" s="12"/>
       <c r="C42" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D42" s="9">
+      <c r="D42" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="10"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="12" t="s">
+      <c r="A43" s="16"/>
+      <c r="B43" s="13"/>
+      <c r="C43" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D43" s="13">
+      <c r="D43" s="7">
         <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="5">
+      <c r="B44" s="11">
         <v>0.12</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D44" s="7">
+      <c r="D44" s="4">
         <v>0.03</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="8"/>
-      <c r="B45" s="3"/>
+      <c r="A45" s="15"/>
+      <c r="B45" s="12"/>
       <c r="C45" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D45" s="9">
+      <c r="D45" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="8"/>
-      <c r="B46" s="3"/>
+      <c r="A46" s="15"/>
+      <c r="B46" s="12"/>
       <c r="C46" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D46" s="9">
+      <c r="D46" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="8"/>
-      <c r="B47" s="3"/>
+      <c r="A47" s="15"/>
+      <c r="B47" s="12"/>
       <c r="C47" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D47" s="9">
+      <c r="D47" s="5">
         <v>0.03</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="8"/>
-      <c r="B48" s="3"/>
+      <c r="A48" s="15"/>
+      <c r="B48" s="12"/>
       <c r="C48" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D48" s="9">
+      <c r="D48" s="5">
         <v>0.02</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="10"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="12" t="s">
+      <c r="A49" s="16"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D49" s="13">
+      <c r="D49" s="7">
         <v>0.03</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B50" s="5">
+      <c r="B50" s="11">
         <v>1.3</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D50" s="7">
+      <c r="D50" s="4">
         <v>0.26</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="8"/>
-      <c r="B51" s="3"/>
+      <c r="A51" s="15"/>
+      <c r="B51" s="12"/>
       <c r="C51" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D51" s="9">
+      <c r="D51" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="8"/>
-      <c r="B52" s="3"/>
+      <c r="A52" s="15"/>
+      <c r="B52" s="12"/>
       <c r="C52" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D52" s="9">
+      <c r="D52" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="8"/>
-      <c r="B53" s="3"/>
+      <c r="A53" s="15"/>
+      <c r="B53" s="12"/>
       <c r="C53" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D53" s="5">
         <v>0.23</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="8"/>
-      <c r="B54" s="3"/>
+      <c r="A54" s="15"/>
+      <c r="B54" s="12"/>
       <c r="C54" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="5">
         <v>0.17</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="10"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="12" t="s">
+      <c r="A55" s="16"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D55" s="13">
+      <c r="D55" s="7">
         <v>0.22</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
+      <c r="A56" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="B56" s="5">
+      <c r="B56" s="11">
         <v>1.41</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D56" s="7">
+      <c r="D56" s="4">
         <v>0.27</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="8"/>
-      <c r="B57" s="3"/>
+      <c r="A57" s="15"/>
+      <c r="B57" s="12"/>
       <c r="C57" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="8"/>
-      <c r="B58" s="3"/>
+      <c r="A58" s="15"/>
+      <c r="B58" s="12"/>
       <c r="C58" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="5">
         <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="8"/>
-      <c r="B59" s="3"/>
+      <c r="A59" s="15"/>
+      <c r="B59" s="12"/>
       <c r="C59" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D59" s="9">
+      <c r="D59" s="5">
         <v>0.25</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="8"/>
-      <c r="B60" s="3"/>
+      <c r="A60" s="15"/>
+      <c r="B60" s="12"/>
       <c r="C60" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="5">
         <v>0.22</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="10"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="12" t="s">
+      <c r="A61" s="16"/>
+      <c r="B61" s="13"/>
+      <c r="C61" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D61" s="13">
+      <c r="D61" s="7">
         <v>0.25</v>
       </c>
     </row>
@@ -1902,16 +1902,17 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A2:A7"/>
+    <mergeCell ref="B2:B7"/>
+    <mergeCell ref="B14:B19"/>
+    <mergeCell ref="B20:B25"/>
+    <mergeCell ref="B26:B31"/>
+    <mergeCell ref="B32:B37"/>
     <mergeCell ref="B50:B55"/>
     <mergeCell ref="B56:B61"/>
     <mergeCell ref="A44:A49"/>
     <mergeCell ref="A56:A61"/>
     <mergeCell ref="B8:B13"/>
-    <mergeCell ref="B2:B7"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B25"/>
-    <mergeCell ref="B26:B31"/>
-    <mergeCell ref="B32:B37"/>
     <mergeCell ref="B38:B43"/>
     <mergeCell ref="B44:B49"/>
     <mergeCell ref="A50:A55"/>
@@ -1921,7 +1922,6 @@
     <mergeCell ref="A26:A31"/>
     <mergeCell ref="A32:A37"/>
     <mergeCell ref="A38:A43"/>
-    <mergeCell ref="A2:A7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added new info, made a few new graphs and did various text fixes for result Excel files
</commit_message>
<xml_diff>
--- a/results/0_excel_files/active_attack_results.xlsx
+++ b/results/0_excel_files/active_attack_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Bakalaura Darbs\!Code\Bakalaura_darbs\results\0_excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB6944-A66A-4166-A5AF-22F5098A6419}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22630CA9-3C18-4484-824B-A2D735629297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1CF9389B-EC12-4777-A84E-B567E82B38F5}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="19">
   <si>
     <t>Active stego-attack type</t>
   </si>
@@ -29,24 +29,6 @@
   </si>
   <si>
     <t>01_insert_attack</t>
-  </si>
-  <si>
-    <t>stego_method_1</t>
-  </si>
-  <si>
-    <t>stego_method_2</t>
-  </si>
-  <si>
-    <t>stego_method_3</t>
-  </si>
-  <si>
-    <t>stego_method_4</t>
-  </si>
-  <si>
-    <t>stego_method_5</t>
-  </si>
-  <si>
-    <t>stego_method_6</t>
   </si>
   <si>
     <t>02_delete_attack</t>
@@ -81,12 +63,27 @@
   <si>
     <t>Total attack time lapse (min.sec)</t>
   </si>
+  <si>
+    <t>hide_in_text</t>
+  </si>
+  <si>
+    <t>modify_RGB_color_ch</t>
+  </si>
+  <si>
+    <t>unispace</t>
+  </si>
+  <si>
+    <t>NOT USED</t>
+  </si>
+  <si>
+    <t>unicode_homoglyphs</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -240,12 +237,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="186"/>
+    </font>
+    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="186"/>
     </font>
   </fonts>
   <fills count="33">
@@ -811,49 +815,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1234,663 +1238,663 @@
   <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="9" t="s">
+    <row r="1" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D1" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="11">
         <v>1.05</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="4">
+      <c r="C2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="6">
         <v>0.19</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>
       <c r="B3" s="12"/>
-      <c r="C3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="12"/>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D4" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5">
+      <c r="C5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="8">
         <v>0.17</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="15"/>
       <c r="B6" s="12"/>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="5">
+      <c r="C6" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="8">
         <v>0.11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16"/>
       <c r="B7" s="13"/>
-      <c r="C7" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="7">
+      <c r="C7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="10">
         <v>0.16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B8" s="11">
         <v>1.04</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="4">
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="6">
         <v>0.18</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="12"/>
-      <c r="C9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D9" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C9" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="12"/>
-      <c r="C10" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="12"/>
-      <c r="C11" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="5">
+      <c r="C11" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="8">
         <v>0.16</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="12"/>
-      <c r="C12" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="5">
+      <c r="C12" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="8">
         <v>0.11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16"/>
       <c r="B13" s="13"/>
-      <c r="C13" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D13" s="7">
+      <c r="C13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="10">
         <v>0.16</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B14" s="11">
         <v>1.05</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" s="4">
+      <c r="C14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="6">
         <v>0.19</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="12"/>
-      <c r="C15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D15" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="12"/>
-      <c r="C16" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D16" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="12"/>
-      <c r="C17" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="5">
+      <c r="C17" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="8">
         <v>0.17</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="12"/>
-      <c r="C18" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D18" s="5">
+      <c r="C18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" s="8">
         <v>0.11</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
       <c r="B19" s="13"/>
-      <c r="C19" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D19" s="7">
+      <c r="C19" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="10">
         <v>0.16</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="14" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B20" s="11">
         <v>5.29</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D20" s="4">
+      <c r="C20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="6">
         <v>1.34</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="12"/>
-      <c r="C21" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D21" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C21" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="12"/>
-      <c r="C22" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C22" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="12"/>
-      <c r="C23" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="5">
+      <c r="C23" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="8">
         <v>1.31</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="5">
+      <c r="C24" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="8">
         <v>0.59</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="16"/>
       <c r="B25" s="13"/>
-      <c r="C25" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="7">
+      <c r="C25" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="10">
         <v>1.24</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="14" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="B26" s="11">
         <v>15.4</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D26" s="4">
+      <c r="C26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="6">
         <v>4.2</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="15"/>
       <c r="B27" s="12"/>
-      <c r="C27" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D27" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C27" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="12"/>
-      <c r="C28" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C28" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="15"/>
       <c r="B29" s="12"/>
-      <c r="C29" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="5">
+      <c r="C29" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="8">
         <v>4.18</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="15"/>
       <c r="B30" s="12"/>
-      <c r="C30" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="5">
+      <c r="C30" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D30" s="8">
         <v>2.34</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="16"/>
       <c r="B31" s="13"/>
-      <c r="C31" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D31" s="7">
+      <c r="C31" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="10">
         <v>4.26</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="B32" s="11">
         <v>1.1499999999999999</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D32" s="4">
+      <c r="C32" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="6">
         <v>0.23</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="15"/>
       <c r="B33" s="12"/>
-      <c r="C33" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D33" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C33" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="15"/>
       <c r="B34" s="12"/>
-      <c r="C34" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C34" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="15"/>
       <c r="B35" s="12"/>
-      <c r="C35" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="5">
+      <c r="C35" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D35" s="8">
         <v>0.19</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="15"/>
       <c r="B36" s="12"/>
-      <c r="C36" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D36" s="5">
+      <c r="C36" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="8">
         <v>0.15</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="16"/>
       <c r="B37" s="13"/>
-      <c r="C37" s="6" t="s">
+      <c r="C37" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="10">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="7">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
+      <c r="B38" s="11">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B38" s="11">
-        <v>0</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D38" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D38" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="15"/>
       <c r="B39" s="12"/>
-      <c r="C39" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D39" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C39" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D39" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="15"/>
       <c r="B40" s="12"/>
-      <c r="C40" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C40" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D40" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="15"/>
       <c r="B41" s="12"/>
-      <c r="C41" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D41" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C41" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D41" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="15"/>
       <c r="B42" s="12"/>
-      <c r="C42" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C42" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D42" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="16"/>
       <c r="B43" s="13"/>
-      <c r="C43" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="14" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B44" s="11">
         <v>0.12</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D44" s="4">
+      <c r="C44" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="6">
         <v>0.03</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="15"/>
       <c r="B45" s="12"/>
-      <c r="C45" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D45" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C45" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D45" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="15"/>
       <c r="B46" s="12"/>
-      <c r="C46" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D46" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C46" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="15"/>
       <c r="B47" s="12"/>
-      <c r="C47" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" s="5">
+      <c r="C47" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D47" s="8">
         <v>0.03</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="15"/>
       <c r="B48" s="12"/>
-      <c r="C48" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D48" s="5">
+      <c r="C48" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D48" s="8">
         <v>0.02</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="16"/>
       <c r="B49" s="13"/>
-      <c r="C49" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D49" s="7">
+      <c r="C49" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" s="10">
         <v>0.03</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="14" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="B50" s="11">
         <v>1.3</v>
       </c>
-      <c r="C50" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D50" s="4">
+      <c r="C50" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" s="6">
         <v>0.26</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="15"/>
       <c r="B51" s="12"/>
-      <c r="C51" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D51" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C51" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D51" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="15"/>
       <c r="B52" s="12"/>
-      <c r="C52" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D52" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C52" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D52" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="15"/>
       <c r="B53" s="12"/>
-      <c r="C53" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D53" s="5">
+      <c r="C53" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D53" s="8">
         <v>0.23</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="15"/>
       <c r="B54" s="12"/>
-      <c r="C54" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D54" s="5">
+      <c r="C54" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D54" s="8">
         <v>0.17</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="16"/>
       <c r="B55" s="13"/>
-      <c r="C55" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D55" s="7">
+      <c r="C55" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D55" s="10">
         <v>0.22</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="14" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B56" s="11">
         <v>1.41</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="D56" s="4">
+      <c r="C56" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" s="6">
         <v>0.27</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="15"/>
       <c r="B57" s="12"/>
-      <c r="C57" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D57" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C57" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D57" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="15"/>
       <c r="B58" s="12"/>
-      <c r="C58" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D58" s="5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C58" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D58" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="15"/>
       <c r="B59" s="12"/>
-      <c r="C59" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D59" s="5">
+      <c r="C59" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D59" s="8">
         <v>0.25</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="15"/>
       <c r="B60" s="12"/>
-      <c r="C60" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D60" s="5">
+      <c r="C60" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D60" s="8">
         <v>0.22</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="16"/>
       <c r="B61" s="13"/>
-      <c r="C61" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="D61" s="7">
+      <c r="C61" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="10">
         <v>0.25</v>
       </c>
     </row>
@@ -1907,19 +1911,19 @@
     <mergeCell ref="B14:B19"/>
     <mergeCell ref="B20:B25"/>
     <mergeCell ref="B26:B31"/>
+    <mergeCell ref="B8:B13"/>
+    <mergeCell ref="A8:A13"/>
+    <mergeCell ref="A14:A19"/>
+    <mergeCell ref="A20:A25"/>
+    <mergeCell ref="A26:A31"/>
     <mergeCell ref="B32:B37"/>
     <mergeCell ref="B50:B55"/>
     <mergeCell ref="B56:B61"/>
     <mergeCell ref="A44:A49"/>
     <mergeCell ref="A56:A61"/>
-    <mergeCell ref="B8:B13"/>
     <mergeCell ref="B38:B43"/>
     <mergeCell ref="B44:B49"/>
     <mergeCell ref="A50:A55"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="A26:A31"/>
     <mergeCell ref="A32:A37"/>
     <mergeCell ref="A38:A43"/>
   </mergeCells>

</xml_diff>

<commit_message>
Unified all result Excel files into 3 files
</commit_message>
<xml_diff>
--- a/results/0_excel_files/active_attack_results.xlsx
+++ b/results/0_excel_files/active_attack_results.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Bakalaura Darbs\!Code\Bakalaura_darbs\results\0_excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22630CA9-3C18-4484-824B-A2D735629297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D192152-EA43-4207-BD94-C648DA7D54F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1CF9389B-EC12-4777-A84E-B567E82B38F5}"/>
   </bookViews>
   <sheets>
-    <sheet name="all_attacks_transposed" sheetId="1" r:id="rId1"/>
+    <sheet name="all_attacks_time" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>

</xml_diff>

<commit_message>
Updated the final Excel file results
</commit_message>
<xml_diff>
--- a/results/0_excel_files/active_attack_results.xlsx
+++ b/results/0_excel_files/active_attack_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\Bakalaura Darbs\!Code\Bakalaura_darbs\results\0_excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D192152-EA43-4207-BD94-C648DA7D54F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{701EA23A-2369-4687-B623-AB9B3BD41FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1CF9389B-EC12-4777-A84E-B567E82B38F5}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="18">
   <si>
     <t>Active stego-attack type</t>
   </si>
@@ -58,12 +58,6 @@
     <t>10_document_inspector_attack</t>
   </si>
   <si>
-    <t>Attack time for each stego-file data set (min.sec)</t>
-  </si>
-  <si>
-    <t>Total attack time lapse (min.sec)</t>
-  </si>
-  <si>
     <t>hide_in_text</t>
   </si>
   <si>
@@ -73,10 +67,15 @@
     <t>unispace</t>
   </si>
   <si>
-    <t>NOT USED</t>
+    <t>unicode_homoglyphs</t>
   </si>
   <si>
-    <t>unicode_homoglyphs</t>
+    <t>Attack time for each 
+stego-file data set (min.sec)</t>
+  </si>
+  <si>
+    <t>Total attack 
+time lapse (min.sec)</t>
   </si>
 </sst>
 </file>
@@ -575,7 +574,20 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
@@ -593,6 +605,124 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -603,33 +733,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -639,127 +750,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -810,9 +801,42 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -824,41 +848,11 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1238,664 +1232,464 @@
   <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>13</v>
+      <c r="B1" s="17" t="s">
+        <v>17</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="10">
+        <v>1.07</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="11">
-        <v>1.05</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="14"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="7">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="14"/>
+      <c r="B4" s="11"/>
+      <c r="C4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="6">
-        <v>0.19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D4" s="7">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="15"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="9">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="10">
+        <v>1.05</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="5">
         <v>0.17</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="8">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="16"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="10">
+    <row r="7" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="14"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="7">
         <v>0.16</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" s="11">
-        <v>1.04</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="A8" s="14"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="6">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D8" s="7">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="15"/>
       <c r="B9" s="12"/>
-      <c r="C9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="8">
-        <v>0</v>
+      <c r="C9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0.15</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="12"/>
-      <c r="C10" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="8">
-        <v>0</v>
+      <c r="A10" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B10" s="10">
+        <v>1.05</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0.17</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="15"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="7" t="s">
+      <c r="A11" s="14"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D11" s="7">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="14"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="7">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="8">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="8">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="16"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="10">
-        <v>0.16</v>
+      <c r="D13" s="9">
+        <v>0.15</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="B14" s="11">
-        <v>1.05</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="A14" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="10">
+        <v>2.19</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="14"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="7">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="14"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="6">
-        <v>0.19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D15" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D16" s="7">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="15"/>
       <c r="B17" s="12"/>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="8">
-        <v>0.17</v>
+      <c r="D17" s="9">
+        <v>0.34</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" s="8">
-        <v>0.11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="16"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="10">
-        <v>0.16</v>
+      <c r="A18" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B18" s="10">
+        <v>17.170000000000002</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="5">
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="14"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="7">
+        <v>4.18</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="11">
-        <v>5.29</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="A20" s="14"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="6">
-        <v>1.34</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D20" s="7">
+        <v>4.13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="15"/>
       <c r="B21" s="12"/>
-      <c r="C21" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D21" s="8">
+      <c r="C21" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="9">
+        <v>4.22</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="10">
+        <v>1.27</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="5">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="14"/>
+      <c r="B23" s="11"/>
+      <c r="C23" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D23" s="7">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="14"/>
+      <c r="B24" s="11"/>
+      <c r="C24" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="7">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="15"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="9">
+        <v>0.19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" s="10">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D22" s="8">
+      <c r="C26" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="5">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="15"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D23" s="8">
-        <v>1.31</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D24" s="8">
-        <v>0.59</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="16"/>
-      <c r="B25" s="13"/>
-      <c r="C25" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="10">
-        <v>1.24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="B26" s="11">
-        <v>15.4</v>
-      </c>
-      <c r="C26" s="5" t="s">
+    <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="14"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="14"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="6">
-        <v>4.2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D27" s="8">
+      <c r="D28" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D28" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="15"/>
       <c r="B29" s="12"/>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D29" s="8">
-        <v>4.18</v>
+      <c r="D29" s="9">
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D30" s="8">
-        <v>2.34</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="16"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D31" s="10">
-        <v>4.26</v>
+      <c r="A30" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B30" s="10">
+        <v>0.15</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="5">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="14"/>
+      <c r="B31" s="11"/>
+      <c r="C31" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" s="7">
+        <v>0.04</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
-        <v>7</v>
-      </c>
-      <c r="B32" s="11">
-        <v>1.1499999999999999</v>
-      </c>
-      <c r="C32" s="5" t="s">
+      <c r="A32" s="14"/>
+      <c r="B32" s="11"/>
+      <c r="C32" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="6">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D32" s="7">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="15"/>
       <c r="B33" s="12"/>
-      <c r="C33" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D33" s="8">
-        <v>0</v>
+      <c r="C33" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D33" s="9">
+        <v>0.03</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A34" s="15"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D34" s="8">
-        <v>0</v>
+      <c r="A34" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B34" s="10">
+        <v>1.35</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="5">
+        <v>0.26</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A35" s="15"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="7" t="s">
+      <c r="A35" s="14"/>
+      <c r="B35" s="11"/>
+      <c r="C35" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="7">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="14"/>
+      <c r="B36" s="11"/>
+      <c r="C36" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="7">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="15"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D35" s="8">
-        <v>0.19</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D36" s="8">
-        <v>0.15</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="16"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="10">
-        <v>0.17</v>
+      <c r="D37" s="9">
+        <v>0.21</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="B38" s="11">
-        <v>0</v>
-      </c>
-      <c r="C38" s="5" t="s">
+      <c r="A38" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="10">
+        <v>1.59</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" s="5">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="14"/>
+      <c r="B39" s="11"/>
+      <c r="C39" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" s="7">
+        <v>0.31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="14"/>
+      <c r="B40" s="11"/>
+      <c r="C40" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D38" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A39" s="15"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D39" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="15"/>
-      <c r="B40" s="12"/>
-      <c r="C40" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D40" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D40" s="7">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="15"/>
       <c r="B41" s="12"/>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D41" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="15"/>
-      <c r="B42" s="12"/>
-      <c r="C42" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D42" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="16"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D43" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="B44" s="11">
-        <v>0.12</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D44" s="6">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
-      <c r="B45" s="12"/>
-      <c r="C45" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D45" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="12"/>
-      <c r="C46" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A47" s="15"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D47" s="8">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A48" s="15"/>
-      <c r="B48" s="12"/>
-      <c r="C48" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D48" s="8">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="16"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D49" s="10">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B50" s="11">
-        <v>1.3</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="6">
+      <c r="D41" s="9">
         <v>0.26</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A51" s="15"/>
-      <c r="B51" s="12"/>
-      <c r="C51" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D51" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A52" s="15"/>
-      <c r="B52" s="12"/>
-      <c r="C52" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D52" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="15"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D53" s="8">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="15"/>
-      <c r="B54" s="12"/>
-      <c r="C54" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D54" s="8">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="16"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D55" s="10">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="B56" s="11">
-        <v>1.41</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D56" s="6">
-        <v>0.27</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="15"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D57" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A58" s="15"/>
-      <c r="B58" s="12"/>
-      <c r="C58" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D58" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="15"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D59" s="8">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A60" s="15"/>
-      <c r="B60" s="12"/>
-      <c r="C60" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D60" s="8">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="16"/>
-      <c r="B61" s="13"/>
-      <c r="C61" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D61" s="10">
-        <v>0.25</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
@@ -1906,26 +1700,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A2:A7"/>
-    <mergeCell ref="B2:B7"/>
-    <mergeCell ref="B14:B19"/>
-    <mergeCell ref="B20:B25"/>
-    <mergeCell ref="B26:B31"/>
-    <mergeCell ref="B8:B13"/>
-    <mergeCell ref="A8:A13"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="A20:A25"/>
-    <mergeCell ref="A26:A31"/>
-    <mergeCell ref="B32:B37"/>
-    <mergeCell ref="B50:B55"/>
-    <mergeCell ref="B56:B61"/>
-    <mergeCell ref="A44:A49"/>
-    <mergeCell ref="A56:A61"/>
-    <mergeCell ref="B38:B43"/>
-    <mergeCell ref="B44:B49"/>
-    <mergeCell ref="A50:A55"/>
-    <mergeCell ref="A32:A37"/>
-    <mergeCell ref="A38:A43"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="A38:A41"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A22:A25"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A14:A17"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A6:A9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>